<commit_message>
fix(reference-data): restore 37 more localities and correct city jurisdictions
</commit_message>
<xml_diff>
--- a/workspace/import-sources/universities/stage-1/South_America_Universities_Import_English_12_Countries_COMPLETE.xlsx
+++ b/workspace/import-sources/universities/stage-1/South_America_Universities_Import_English_12_Countries_COMPLETE.xlsx
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P868"/>
+  <dimension ref="A1:P869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="84" min="1" max="1"/>
@@ -36352,7 +36352,7 @@
       </c>
       <c r="N532" t="inlineStr">
         <is>
-          <t>EC-G</t>
+          <t>EC-SE</t>
         </is>
       </c>
       <c r="O532" t="inlineStr">
@@ -59273,7 +59273,78 @@
         </is>
       </c>
     </row>
-    <row r="869" ht="28" customHeight="1" s="84"/>
+    <row r="869" ht="28" customHeight="1" s="84">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>INS-PER-0028</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Universidad Nacional Agraria de la Selva</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Universidad Nacional Agraria de la Selva</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>PER</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>Tingo María</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>Agricultural University</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L869" t="inlineStr">
+        <is>
+          <t>https://www.sunedu.gob.pe/lista-de-universidades-licenciadas/</t>
+        </is>
+      </c>
+      <c r="M869" t="inlineStr">
+        <is>
+          <t>city_pe_geonames_3691348</t>
+        </is>
+      </c>
+      <c r="N869" t="inlineStr">
+        <is>
+          <t>PE-HUC</t>
+        </is>
+      </c>
+      <c r="O869" t="inlineStr">
+        <is>
+          <t>SOURCE_MATCHED</t>
+        </is>
+      </c>
+      <c r="P869" t="inlineStr">
+        <is>
+          <t>REGISTRY_CITY_CORROBORATED_MAIN_CAMPUS_NOT_LIVE_VERIFIED</t>
+        </is>
+      </c>
+    </row>
     <row r="870" ht="28" customHeight="1" s="84"/>
     <row r="871" ht="28" customHeight="1" s="84"/>
     <row r="872" ht="28" customHeight="1" s="84"/>
@@ -60324,7 +60395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60970,17 +61041,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>INS-PER-0028</t>
+          <t>INS-PER-0032</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Universidad Nacional Agraria de la Selva</t>
+          <t>Universidad Nacional Intercultural de Quillabamba</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Universidad Nacional Agraria de la Selva</t>
+          <t>Universidad Nacional Intercultural de Quillabamba</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -60995,12 +61066,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Tingo María</t>
+          <t>Quillabamba</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Agricultural University</t>
+          <t>Intercultural University</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -61032,17 +61103,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>INS-PER-0032</t>
+          <t>INS-PER-0093</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Universidad Nacional Intercultural de Quillabamba</t>
+          <t>Universidad Nacional Autónoma de Huanta</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Universidad Nacional Intercultural de Quillabamba</t>
+          <t>Universidad Nacional Autónoma de Huanta</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -61057,12 +61128,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Quillabamba</t>
+          <t>Huanta</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Intercultural University</t>
+          <t>University</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -61087,39 +61158,39 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
+          <t>OFFICIAL_ADDRESS_GEOGRAPHY_AMBIGUOUS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>INS-PER-0093</t>
+          <t>INS-VEN-0020</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Universidad Nacional Autónoma de Huanta</t>
+          <t>Universidad Nacional Experimental Sur del Lago Jesús María Semprum</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Universidad Nacional Autónoma de Huanta</t>
+          <t>Universidad Nacional Experimental Sur del Lago Jesús María Semprum</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>PER</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Huanta</t>
+          <t>Santa Bárbara del Zulia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -61137,9 +61208,14 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://www.unesur.edu.ve/</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.sunedu.gob.pe/lista-de-universidades-licenciadas/</t>
+          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -61149,24 +61225,24 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>OFFICIAL_ADDRESS_GEOGRAPHY_AMBIGUOUS</t>
+          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>INS-VEN-0020</t>
+          <t>INS-VEN-0032</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Universidad Nacional Experimental Sur del Lago Jesús María Semprum</t>
+          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Universidad Nacional Experimental Sur del Lago Jesús María Semprum</t>
+          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -61181,12 +61257,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Santa Bárbara del Zulia</t>
+          <t>Mantecal</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Technical University</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -61197,11 +61273,6 @@
       <c r="J14" t="inlineStr">
         <is>
           <t>Active</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>https://www.unesur.edu.ve/</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -61223,17 +61294,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INS-VEN-0032</t>
+          <t>INS-VEN-0043</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
+          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
+          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -61246,14 +61317,9 @@
           <t>VEN</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Mantecal</t>
-        </is>
-      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Technical University</t>
+          <t>Agricultural University</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -61277,63 +61343,6 @@
         </is>
       </c>
       <c r="P15" t="inlineStr">
-        <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>INS-VEN-0043</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Venezuela</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>VEN</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Agricultural University</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>REVIEW_REQUIRED</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
         <is>
           <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
         </is>

</xml_diff>

<commit_message>
fix(reference-data): verify 68 more university city bindings
</commit_message>
<xml_diff>
--- a/workspace/import-sources/universities/stage-1/South_America_Universities_Import_English_12_Countries_COMPLETE.xlsx
+++ b/workspace/import-sources/universities/stage-1/South_America_Universities_Import_English_12_Countries_COMPLETE.xlsx
@@ -849,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P873"/>
+  <dimension ref="A1:P875"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="84" min="1" max="1"/>
@@ -59638,8 +59638,140 @@
         </is>
       </c>
     </row>
-    <row r="874" ht="28" customHeight="1" s="84"/>
-    <row r="875" ht="28" customHeight="1" s="84"/>
+    <row r="874" ht="28" customHeight="1" s="84">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>INS-ARG-0068</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Universidad Provincial de Laguna Blanca</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Universidad Provincial de Laguna Blanca</t>
+        </is>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>ARG</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>Laguna Blanca</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L874" t="inlineStr">
+        <is>
+          <t>https://www.argentina.gob.ar/educacion/universidades/informacion-universitaria/instituciones-universitarias</t>
+        </is>
+      </c>
+      <c r="M874" t="inlineStr">
+        <is>
+          <t>city_ar_official_laguna_blanca</t>
+        </is>
+      </c>
+      <c r="N874" t="inlineStr">
+        <is>
+          <t>AR-P</t>
+        </is>
+      </c>
+      <c r="O874" t="inlineStr">
+        <is>
+          <t>SOURCE_MATCHED</t>
+        </is>
+      </c>
+    </row>
+    <row r="875" ht="28" customHeight="1" s="84">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>INS-PRY-0038</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Universidad Nacional de Canindeyú</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Universidad Nacional de Canindeyú</t>
+        </is>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>PRY</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>Salto del Guaira</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="L875" t="inlineStr">
+        <is>
+          <t>https://cones.gov.py/universidades/</t>
+        </is>
+      </c>
+      <c r="M875" t="inlineStr">
+        <is>
+          <t>city_py_salto_del_guaira</t>
+        </is>
+      </c>
+      <c r="N875" t="inlineStr">
+        <is>
+          <t>PY-14</t>
+        </is>
+      </c>
+      <c r="O875" t="inlineStr">
+        <is>
+          <t>SOURCE_MATCHED</t>
+        </is>
+      </c>
+    </row>
     <row r="876" ht="28" customHeight="1" s="84"/>
     <row r="877" ht="28" customHeight="1" s="84"/>
     <row r="878" ht="28" customHeight="1" s="84"/>
@@ -60684,7 +60816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -60834,32 +60966,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INS-ARG-0068</t>
+          <t>INS-BOL-0008</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Universidad Provincial de Laguna Blanca</t>
+          <t>Universidad Nacional Siglo XX</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Universidad Provincial de Laguna Blanca</t>
+          <t>Universidad Nacional Siglo XX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ARG</t>
+          <t>BOL</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Laguna Blanca</t>
+          <t>Llallagua</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -60879,7 +61011,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://www.argentina.gob.ar/educacion/universidades/informacion-universitaria/instituciones-universitarias</t>
+          <t>https://ceub.edu.bo/universidades-del-sistema/ | https://dgesu.minedu.gob.bo/</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -60896,17 +61028,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INS-BOL-0008</t>
+          <t>INS-BOL-0011</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Universidad Nacional Siglo XX</t>
+          <t>Universidad Indígena Boliviana Aymara Túpac Katari</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Universidad Nacional Siglo XX</t>
+          <t>Universidad Indígena Boliviana Aymara Túpac Katari</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -60921,7 +61053,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Llallagua</t>
+          <t>Warisata</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -60958,17 +61090,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INS-BOL-0011</t>
+          <t>INS-BOL-0013</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Universidad Indígena Boliviana Aymara Túpac Katari</t>
+          <t>Universidad Indígena Boliviana Guaraní y Pueblos de Tierras Bajas Apiaguaiki Tüpa</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Universidad Indígena Boliviana Aymara Túpac Katari</t>
+          <t>Universidad Indígena Boliviana Guaraní y Pueblos de Tierras Bajas Apiaguaiki Tüpa</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -60983,7 +61115,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Warisata</t>
+          <t>Kuruyuki</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -61020,32 +61152,32 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>INS-BOL-0013</t>
+          <t>INS-BRA-0133</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Universidad Indígena Boliviana Guaraní y Pueblos de Tierras Bajas Apiaguaiki Tüpa</t>
+          <t>Universidade do Grande Rio</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Universidad Indígena Boliviana Guaraní y Pueblos de Tierras Bajas Apiaguaiki Tüpa</t>
+          <t>Universidade do Grande Rio</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BOL</t>
+          <t>BRA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Kuruyuki</t>
+          <t>Duque de Caxias</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -61055,7 +61187,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Public</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -61065,7 +61197,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://ceub.edu.bo/universidades-del-sistema/ | https://dgesu.minedu.gob.bo/</t>
+          <t>https://emec.mec.gov.br/ | https://www.gov.br/mec/pt-br/politica-regulacao-supervisao-educacao-superior/cadastro-nacional-de-cursos-e-ies</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -61082,32 +61214,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>INS-BRA-0133</t>
+          <t>INS-PRY-0056</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Universidade do Grande Rio</t>
+          <t>Universidad Santa Clara de Asís</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Universidade do Grande Rio</t>
+          <t>Universidad Santa Clara de Asís</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BRA</t>
+          <t>PRY</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Duque de Caxias</t>
+          <t>Caaguazú</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -61127,7 +61259,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://emec.mec.gov.br/ | https://www.gov.br/mec/pt-br/politica-regulacao-supervisao-educacao-superior/cadastro-nacional-de-cursos-e-ies</t>
+          <t>https://cones.gov.py/universidades/</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -61144,37 +61276,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>INS-PRY-0038</t>
+          <t>INS-VEN-0032</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Canindeyú</t>
+          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Canindeyú</t>
+          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PRY</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Saltos del Guairá</t>
+          <t>Mantecal</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Technical University</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -61189,7 +61321,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://cones.gov.py/universidades/</t>
+          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -61206,42 +61338,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INS-PRY-0056</t>
+          <t>INS-VEN-0043</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Universidad Santa Clara de Asís</t>
+          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Universidad Santa Clara de Asís</t>
+          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PRY</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Caaguazú</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Agricultural University</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Private</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -61251,7 +61378,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://cones.gov.py/universidades/</t>
+          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -61260,125 +61387,6 @@
         </is>
       </c>
       <c r="P9" t="inlineStr">
-        <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>INS-VEN-0032</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Universidad Politécnica Territorial del Alto Apure Pedro Camejo</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Venezuela</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>VEN</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Mantecal</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Technical University</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>REVIEW_REQUIRED</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>INS-VEN-0043</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Universidad Campesina de Venezuela Argimiro Gabaldón</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Venezuela</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>VEN</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Agricultural University</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>https://cnu.gob.ve/wp-content/uploads/2024/04/Directorio-CNU-Abril-2024.pdf | https://loeu.opsu.gob.ve/ieu/</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>REVIEW_REQUIRED</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
         <is>
           <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
         </is>

</xml_diff>